<commit_message>
Checked script reproducibility and added processed data for figures
</commit_message>
<xml_diff>
--- a/manuscript_sourcedata/source_data_fig5.xlsx
+++ b/manuscript_sourcedata/source_data_fig5.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yyj/Doc/1_dod_dec25/manu_sourcedata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yyj/Doc/1_dod_dec25/manuscript_sourcedata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F56646-12D1-4343-8169-7CABD24CEB43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF4ECE4-D85B-274C-B583-33AE50596D2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="53120" yWindow="1200" windowWidth="34560" windowHeight="21580" activeTab="4" xr2:uid="{253B514A-1DCE-8746-A201-6795F8FD4B91}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="4" xr2:uid="{253B514A-1DCE-8746-A201-6795F8FD4B91}"/>
   </bookViews>
   <sheets>
     <sheet name="5a" sheetId="10" r:id="rId1"/>
@@ -111,12 +111,6 @@
     <t>ANBL-CHP-Patient2-PT-R-DNA_mixcr_out.clones_TRB</t>
   </si>
   <si>
-    <t>ANBL-SM-907322-T0-M-DNA_mixcr_out.clones_TRB</t>
-  </si>
-  <si>
-    <t>ANBL-SM-907322-T1-M-DNA_mixcr_out.clones_TRB</t>
-  </si>
-  <si>
     <t>CASSVIAETYEQYF</t>
   </si>
   <si>
@@ -126,12 +120,6 @@
     <t>ANBL-CHP-Patient2-PT-R-DNA_mixcr_out.clones_TRA</t>
   </si>
   <si>
-    <t>ANBL-SM-907322-T0-M-DNA_mixcr_out.clones_TRA</t>
-  </si>
-  <si>
-    <t>ANBL-SM-907322-T1-M-DNA_mixcr_out.clones_TRA</t>
-  </si>
-  <si>
     <t>CAAKQAGYSTLTF</t>
   </si>
   <si>
@@ -150,12 +138,6 @@
     <t>ANBL-CHP-Patient2-PT-R-DNA_mixcr_out</t>
   </si>
   <si>
-    <t>ANBL-SM-907322-T0-M-DNA_mixcr_out</t>
-  </si>
-  <si>
-    <t>ANBL-SM-907322-T1-M-DNA_mixcr_out</t>
-  </si>
-  <si>
     <t>ANBL-SM-Patient17-T2-M-DNA_mixcr_out</t>
   </si>
   <si>
@@ -190,6 +172,24 @@
   </si>
   <si>
     <t>a Clone 7</t>
+  </si>
+  <si>
+    <t>ANBL-SM-Patient2-T0-M-DNA_mixcr_out</t>
+  </si>
+  <si>
+    <t>ANBL-SM-Patient2-T1-M-DNA_mixcr_out</t>
+  </si>
+  <si>
+    <t>ANBL-SM-Patient2-T0-M-DNA_mixcr_out.clones_TRA</t>
+  </si>
+  <si>
+    <t>ANBL-SM-Patient2-T1-M-DNA_mixcr_out.clones_TRA</t>
+  </si>
+  <si>
+    <t>ANBL-SM-Patient2-T0-M-DNA_mixcr_out.clones_TRB</t>
+  </si>
+  <si>
+    <t>ANBL-SM-Patient2-T1-M-DNA_mixcr_out.clones_TRB</t>
   </si>
 </sst>
 </file>
@@ -569,16 +569,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -620,7 +620,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C4">
         <v>9.4151358542700694E-3</v>
@@ -637,7 +637,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C5">
         <v>2.8144165336469701E-3</v>
@@ -688,7 +688,7 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C8">
         <v>9.6198127206672396E-3</v>
@@ -705,7 +705,7 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C9">
         <v>4.8727211627320804E-3</v>
@@ -722,7 +722,7 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C10">
         <v>2.2770301386685701E-2</v>
@@ -739,7 +739,7 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C11">
         <v>2.33134503906578E-3</v>
@@ -756,7 +756,7 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C12">
         <v>2.35378396356751E-3</v>
@@ -773,7 +773,7 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C13">
         <v>1.11106443753675E-2</v>
@@ -936,39 +936,39 @@
         <v>11</v>
       </c>
       <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
         <v>31</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" t="s">
         <v>32</v>
       </c>
-      <c r="D1" t="s">
+      <c r="J1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" t="s">
+      <c r="K1" t="s">
         <v>34</v>
-      </c>
-      <c r="F1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B2">
         <v>4.9884231449727999E-3</v>
@@ -1084,21 +1084,21 @@
         <v>11</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="E1" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B2">
         <v>0.161043088139078</v>
@@ -1134,15 +1134,15 @@
         <v>22</v>
       </c>
       <c r="D1" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="E1" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2">
         <v>0.26083598107018302</v>

</xml_diff>